<commit_message>
Update Caesalpinia pulcherrima image and replace S1B & S46 before/after Images
</commit_message>
<xml_diff>
--- a/data/BeforeAndAfter.xlsx
+++ b/data/BeforeAndAfter.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3C698A-A362-456B-81C4-7DD161A8A99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE9965D-9E63-4BE0-AD27-D3FB16365432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="151">
   <si>
     <t>Location Type</t>
   </si>
@@ -270,9 +270,6 @@
   </si>
   <si>
     <t>College of Business Administration</t>
-  </si>
-  <si>
-    <t>https://i.postimg.cc/qR6zJM6N/SA-01-B.jpg</t>
   </si>
   <si>
     <t>S46</t>
@@ -1094,7 +1091,7 @@
         <v>12</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>13</v>
@@ -1166,7 +1163,7 @@
         <v>19</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -1609,7 +1606,7 @@
         <v>56</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="14" t="s">
@@ -1784,10 +1781,10 @@
         <v>9</v>
       </c>
       <c r="B35" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>55</v>
@@ -1796,7 +1793,7 @@
         <v>56</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="G35" s="15"/>
       <c r="H35" s="16" t="s">
@@ -1811,10 +1808,10 @@
         <v>9</v>
       </c>
       <c r="B36" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D36" s="18" t="s">
         <v>55</v>
@@ -1834,10 +1831,10 @@
         <v>9</v>
       </c>
       <c r="B37" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D37" s="18" t="s">
         <v>55</v>
@@ -1857,10 +1854,10 @@
         <v>9</v>
       </c>
       <c r="B38" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D38" s="18" t="s">
         <v>55</v>
@@ -1880,10 +1877,10 @@
         <v>9</v>
       </c>
       <c r="B39" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D39" s="18" t="s">
         <v>55</v>
@@ -1903,10 +1900,10 @@
         <v>9</v>
       </c>
       <c r="B40" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D40" s="18" t="s">
         <v>55</v>
@@ -1926,10 +1923,10 @@
         <v>9</v>
       </c>
       <c r="B41" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C41" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C41" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D41" s="18" t="s">
         <v>55</v>
@@ -1949,10 +1946,10 @@
         <v>9</v>
       </c>
       <c r="B42" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D42" s="18" t="s">
         <v>55</v>
@@ -1972,10 +1969,10 @@
         <v>9</v>
       </c>
       <c r="B43" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D43" s="18" t="s">
         <v>55</v>
@@ -2001,16 +1998,16 @@
         <v>54</v>
       </c>
       <c r="D44" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E44" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="E44" s="20" t="s">
+      <c r="F44" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="H44" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>84</v>
       </c>
       <c r="I44" s="7"/>
     </row>
@@ -2025,13 +2022,13 @@
         <v>54</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F45" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="H45" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>86</v>
       </c>
       <c r="I45" s="7"/>
     </row>
@@ -2046,13 +2043,13 @@
         <v>54</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F46" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H46" s="7" t="s">
         <v>87</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="I46" s="7"/>
     </row>
@@ -2067,13 +2064,13 @@
         <v>54</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F47" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H47" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="I47" s="7"/>
     </row>
@@ -2082,25 +2079,25 @@
         <v>9</v>
       </c>
       <c r="B48" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="D48" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D48" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G48" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I48" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="6" customFormat="1" ht="217.5" x14ac:dyDescent="0.35">
@@ -2108,25 +2105,25 @@
         <v>9</v>
       </c>
       <c r="B49" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C49" s="13" t="s">
-        <v>92</v>
-      </c>
       <c r="D49" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E49" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="F49" s="7" t="s">
+      <c r="H49" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="H49" s="7" t="s">
+      <c r="I49" s="7" t="s">
         <v>99</v>
-      </c>
-      <c r="I49" s="7" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2134,20 +2131,20 @@
         <v>9</v>
       </c>
       <c r="B50" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C50" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C50" s="13" t="s">
-        <v>92</v>
-      </c>
       <c r="D50" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E50" s="12"/>
       <c r="F50" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="H50" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="I50" s="7"/>
     </row>
@@ -2156,20 +2153,20 @@
         <v>9</v>
       </c>
       <c r="B51" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C51" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C51" s="13" t="s">
-        <v>92</v>
-      </c>
       <c r="D51" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E51" s="12"/>
       <c r="F51" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H51" s="7" t="s">
         <v>103</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="I51" s="7"/>
     </row>
@@ -2178,20 +2175,20 @@
         <v>9</v>
       </c>
       <c r="B52" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C52" s="13" t="s">
-        <v>92</v>
-      </c>
       <c r="D52" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E52" s="12"/>
       <c r="F52" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="H52" s="7" t="s">
         <v>105</v>
-      </c>
-      <c r="H52" s="7" t="s">
-        <v>106</v>
       </c>
       <c r="I52" s="7"/>
     </row>
@@ -2200,20 +2197,20 @@
         <v>9</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C53" s="13" t="s">
-        <v>92</v>
-      </c>
       <c r="D53" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E53" s="12"/>
       <c r="F53" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="H53" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="H53" s="7" t="s">
-        <v>108</v>
       </c>
       <c r="I53" s="7"/>
     </row>
@@ -2222,25 +2219,25 @@
         <v>9</v>
       </c>
       <c r="B54" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="D54" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="E54" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F54" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E54" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="F54" s="3" t="s">
+      <c r="H54" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H54" s="3" t="s">
+      <c r="I54" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2248,19 +2245,19 @@
         <v>9</v>
       </c>
       <c r="B55" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C55" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="D55" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D55" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="F55" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H55" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2268,19 +2265,19 @@
         <v>9</v>
       </c>
       <c r="B56" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C56" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="D56" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D56" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="F56" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H56" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2288,19 +2285,19 @@
         <v>9</v>
       </c>
       <c r="B57" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C57" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="D57" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="F57" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H57" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="H57" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2308,19 +2305,19 @@
         <v>9</v>
       </c>
       <c r="B58" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C58" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="D58" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D58" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="F58" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="H58" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" ht="203" x14ac:dyDescent="0.35">
@@ -2328,25 +2325,25 @@
         <v>9</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C59" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="D59" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D59" s="6" t="s">
+      <c r="E59" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="F59" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E59" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="F59" s="7" t="s">
+      <c r="H59" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="H59" s="7" t="s">
+      <c r="I59" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="I59" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2354,19 +2351,19 @@
         <v>9</v>
       </c>
       <c r="B60" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C60" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C60" s="13" t="s">
+      <c r="D60" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D60" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="F60" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2374,19 +2371,19 @@
         <v>9</v>
       </c>
       <c r="B61" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="D61" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D61" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="F61" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="H61" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="H61" s="7" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2394,19 +2391,19 @@
         <v>9</v>
       </c>
       <c r="B62" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C62" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="D62" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D62" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="F62" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H62" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="H62" s="7" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:9" s="4" customFormat="1" ht="203" x14ac:dyDescent="0.35">
@@ -2414,25 +2411,25 @@
         <v>9</v>
       </c>
       <c r="B63" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="D63" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E63" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D63" s="4" t="s">
+      <c r="F63" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E63" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="F63" s="3" t="s">
+      <c r="H63" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H63" s="3" t="s">
+      <c r="I63" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="64" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2440,19 +2437,19 @@
         <v>9</v>
       </c>
       <c r="B64" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C64" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C64" s="10" t="s">
-        <v>145</v>
-      </c>
       <c r="D64" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2460,19 +2457,19 @@
         <v>9</v>
       </c>
       <c r="B65" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C65" s="10" t="s">
-        <v>145</v>
-      </c>
       <c r="D65" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F65" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="H65" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="66" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2480,19 +2477,19 @@
         <v>9</v>
       </c>
       <c r="B66" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C66" s="10" t="s">
-        <v>145</v>
-      </c>
       <c r="D66" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F66" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="H66" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="67" spans="1:9" s="6" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
@@ -2509,13 +2506,13 @@
         <v>11</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F67" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="H67" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>121</v>
       </c>
       <c r="I67" s="7"/>
     </row>
@@ -2533,10 +2530,10 @@
         <v>11</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H68" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2553,10 +2550,10 @@
         <v>11</v>
       </c>
       <c r="F69" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H69" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="H69" s="7" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="70" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -2573,10 +2570,10 @@
         <v>11</v>
       </c>
       <c r="F70" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="H70" s="7" t="s">
         <v>126</v>
-      </c>
-      <c r="H70" s="7" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="71" spans="1:9" s="4" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
@@ -2584,26 +2581,26 @@
         <v>9</v>
       </c>
       <c r="B71" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C71" s="10" t="s">
+      <c r="D71" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D71" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F71" s="3" t="s">
+      <c r="G71" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="H71" s="3"/>
       <c r="I71" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="72" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2611,42 +2608,42 @@
         <v>9</v>
       </c>
       <c r="B72" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C72" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C72" s="10" t="s">
-        <v>129</v>
-      </c>
       <c r="D72" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="73" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A73" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>53</v>
       </c>
       <c r="C73" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D73" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="E73" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="F73" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="E73" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="F73" s="7" t="s">
+      <c r="G73" s="7" t="s">
         <v>137</v>
-      </c>
-      <c r="G73" s="7" t="s">
-        <v>138</v>
       </c>
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
@@ -2656,22 +2653,22 @@
         <v>9</v>
       </c>
       <c r="B74" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C74" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C74" s="9" t="s">
-        <v>96</v>
-      </c>
       <c r="D74" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F74" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G74" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>140</v>
       </c>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>

</xml_diff>